<commit_message>
Latest generated outputs 2026-05-12
</commit_message>
<xml_diff>
--- a/generated/spreadsheet/full-planning-permission-full.xlsx
+++ b/generated/spreadsheet/full-planning-permission-full.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I211"/>
+  <dimension ref="A1:I210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -3943,24 +3943,20 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Building elements[]</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>Building element type</t>
-        </is>
-      </c>
+          <t>Proposal material details</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr"/>
       <c r="E108" s="2" t="inlineStr"/>
       <c r="F108" s="2" t="inlineStr"/>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>The part of building the materials relate to, such as walls, roofs, windows, or doors</t>
+          <t>Whether the proposal involves material details that need to be provided</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
@@ -3979,24 +3975,24 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Existing materials</t>
+          <t>Building element type</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr"/>
       <c r="F109" s="2" t="inlineStr"/>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Description of the materials currently used for this building element</t>
+          <t>The part of building the materials relate to, such as walls, roofs, windows, or doors</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -4010,14 +4006,14 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Proposed materials</t>
+          <t>Existing materials</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr"/>
       <c r="F110" s="2" t="inlineStr"/>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Description of the materials proposed for this building element as part of the development</t>
+          <t>Description of the materials currently used for this building element</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -4041,19 +4037,19 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Materials not applicable</t>
+          <t>Proposed materials</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr"/>
       <c r="F111" s="2" t="inlineStr"/>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>Indicates this building element is not relevant to the application</t>
+          <t>Description of the materials proposed for this building element as part of the development</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr">
@@ -5143,7 +5139,8 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>How waste will be managed on the site</t>
+          <t xml:space="preserve">How waste will be managed on the site
+</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
@@ -5183,7 +5180,7 @@
       <c r="F148" s="2" t="inlineStr"/>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>Whether the proposal involves waste management development</t>
+          <t>Whether the proposal involves any waste management facility that is relevant to the proposal</t>
         </is>
       </c>
       <c r="H148" s="2" t="inlineStr">
@@ -5214,7 +5211,7 @@
       <c r="F149" s="2" t="inlineStr"/>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>Type of waste management facility</t>
+          <t>Type of waste management facility being described in this entry</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
@@ -5238,24 +5235,24 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Total capacity</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr"/>
       <c r="F150" s="2" t="inlineStr"/>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>Whether the facility is not applicable</t>
+          <t>Total capacity of void in cubic metres (or tonnes/litres)</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -5269,24 +5266,24 @@
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Total capacity</t>
+          <t>Unit type</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr"/>
       <c r="F151" s="2" t="inlineStr"/>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>Total capacity of void in cubic metres (or tonnes/litres)</t>
+          <t>Unit for capacity/throughput (e.g. cubic metres, tonnes, litres)</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -5300,24 +5297,24 @@
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Unit type</t>
+          <t>Annual throughput</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr"/>
       <c r="F152" s="2" t="inlineStr"/>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>Unit for capacity/throughput (e.g. cubic metres, tonnes, litres)</t>
+          <t>Maximum annual operational throughput in tonnes/litres</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -5331,24 +5328,24 @@
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Annual throughput</t>
+          <t>Unit type</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr"/>
       <c r="F153" s="2" t="inlineStr"/>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>Maximum annual operational throughput in tonnes/litres</t>
+          <t>Unit for capacity/throughput (e.g. cubic metres, tonnes, litres)</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -5357,24 +5354,24 @@
       <c r="B154" s="2" t="n"/>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Waste management[]</t>
+          <t>Waste streams throughput</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Unit type</t>
+          <t>Municipal</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr"/>
       <c r="F154" s="2" t="inlineStr"/>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>Unit for capacity/throughput (e.g. cubic metres, tonnes, litres)</t>
+          <t>Maximum throughput for municipal waste (annual throughput in tonnes/litres)</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr">
@@ -5393,14 +5390,14 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Construction demolition</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr"/>
       <c r="F155" s="2" t="inlineStr"/>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>Maximum throughput for municipal waste (annual throughput in tonnes/litres)</t>
+          <t>Maximum throughput for construction and demolition waste (annual throughput in tonnes/litres)</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
@@ -5424,14 +5421,14 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>Construction demolition</t>
+          <t>Commercial industrial</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr"/>
       <c r="F156" s="2" t="inlineStr"/>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>Maximum throughput for construction and demolition waste (annual throughput in tonnes/litres)</t>
+          <t>Maximum throughput for commercial and industrial waste (annual throughput in tonnes/litres)</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr">
@@ -5455,14 +5452,14 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>Commercial industrial</t>
+          <t>Hazardous</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr"/>
       <c r="F157" s="2" t="inlineStr"/>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>Maximum throughput for commercial and industrial waste (annual throughput in tonnes/litres)</t>
+          <t>Maximum throughput for hazardous waste (annual throughput in tonnes/litres)</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr">
@@ -5477,50 +5474,46 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n"/>
-      <c r="B158" s="2" t="n"/>
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Description of the proposal</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>What development, works or change of use is proposed</t>
+        </is>
+      </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>Waste streams throughput</t>
-        </is>
-      </c>
-      <c r="D158" s="2" t="inlineStr">
-        <is>
-          <t>Hazardous</t>
-        </is>
-      </c>
+          <t>Proposal description</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr"/>
       <c r="E158" s="2" t="inlineStr"/>
       <c r="F158" s="2" t="inlineStr"/>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>Maximum throughput for hazardous waste (annual throughput in tonnes/litres)</t>
+          <t>A description of what is being proposed, including the development, works, or change of use</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="inlineStr">
-        <is>
-          <t>Description of the proposal</t>
-        </is>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
-        <is>
-          <t>What development, works or change of use is proposed</t>
-        </is>
-      </c>
+      <c r="A159" s="2" t="n"/>
+      <c r="B159" s="2" t="n"/>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Proposal description</t>
+          <t>Proposal started</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr"/>
@@ -5528,12 +5521,12 @@
       <c r="F159" s="2" t="inlineStr"/>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>A description of what is being proposed, including the development, works, or change of use</t>
+          <t>Has any work on the proposal already been started</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I159" s="2" t="inlineStr">
@@ -5547,7 +5540,7 @@
       <c r="B160" s="2" t="n"/>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Proposal started</t>
+          <t>Proposal start date</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr"/>
@@ -5555,17 +5548,17 @@
       <c r="F160" s="2" t="inlineStr"/>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>Has any work on the proposal already been started</t>
+          <t>The date when work on the proposal started, in YYYY-MM-DD format</t>
         </is>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5567,7 @@
       <c r="B161" s="2" t="n"/>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Proposal start date</t>
+          <t>Proposal completed</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr"/>
@@ -5582,17 +5575,17 @@
       <c r="F161" s="2" t="inlineStr"/>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>The date when work on the proposal started, in YYYY-MM-DD format</t>
+          <t>Has any work on the proposal already been completed</t>
         </is>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5594,7 @@
       <c r="B162" s="2" t="n"/>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Proposal completed</t>
+          <t>Proposal completion date</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr"/>
@@ -5609,17 +5602,17 @@
       <c r="F162" s="2" t="inlineStr"/>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>Has any work on the proposal already been completed</t>
+          <t>The date when work on the proposal was completed, in YYYY-MM-DD format</t>
         </is>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -5628,7 +5621,7 @@
       <c r="B163" s="2" t="n"/>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Proposal completion date</t>
+          <t>PIP reference</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr"/>
@@ -5636,12 +5629,12 @@
       <c r="F163" s="2" t="inlineStr"/>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>The date when work on the proposal was completed, in YYYY-MM-DD format</t>
+          <t>Reference number for the Planning in Principle (PIP) application this relates to</t>
         </is>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I163" s="2" t="inlineStr">
@@ -5655,7 +5648,7 @@
       <c r="B164" s="2" t="n"/>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>PIP reference</t>
+          <t>Is public service infrastructure</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr"/>
@@ -5663,26 +5656,34 @@
       <c r="F164" s="2" t="inlineStr"/>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>Reference number for the Planning in Principle (PIP) application this relates to</t>
+          <t>For applications made on or after 1 August 2021, is the proposal for public service infrastructure development</t>
         </is>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n"/>
-      <c r="B165" s="2" t="n"/>
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>Residential units</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Details of the residential units that make up both the current and proposed development.</t>
+        </is>
+      </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Is public service infrastructure</t>
+          <t>Residential unit change</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr"/>
@@ -5690,7 +5691,7 @@
       <c r="F165" s="2" t="inlineStr"/>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>For applications made on or after 1 August 2021, is the proposal for public service infrastructure development</t>
+          <t>Proposal includes the gain, loss or change of use of residential units</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -5705,32 +5706,28 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="inlineStr">
-        <is>
-          <t>Residential units</t>
-        </is>
-      </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>Details of the residential units that make up both the current and proposed development.</t>
-        </is>
-      </c>
+      <c r="A166" s="2" t="n"/>
+      <c r="B166" s="2" t="n"/>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Residential unit change</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="inlineStr"/>
+          <t>Residential unit summary[]</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>Tenure type</t>
+        </is>
+      </c>
       <c r="E166" s="2" t="inlineStr"/>
       <c r="F166" s="2" t="inlineStr"/>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>Proposal includes the gain, loss or change of use of residential units</t>
+          <t>Category of housing tenure</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I166" s="2" t="inlineStr">
@@ -5749,14 +5746,14 @@
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>Tenure type</t>
+          <t>Housing type</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr"/>
       <c r="F167" s="2" t="inlineStr"/>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>Category of housing tenure</t>
+          <t>Type of housing</t>
         </is>
       </c>
       <c r="H167" s="2" t="inlineStr">
@@ -5780,19 +5777,23 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>Housing type</t>
-        </is>
-      </c>
-      <c r="E168" s="2" t="inlineStr"/>
+          <t>Existing unit breakdown[]</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>Units unknown</t>
+        </is>
+      </c>
       <c r="F168" s="2" t="inlineStr"/>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>Type of housing</t>
+          <t>Whether the number of units is unknown</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I168" s="2" t="inlineStr">
@@ -5816,13 +5817,17 @@
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>Units unknown</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr"/>
+          <t>Units per bedroom number[]</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>No bedrooms unknown</t>
+        </is>
+      </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>Whether the number of units is unknown</t>
+          <t>Set to true when counting units where bedroom number is unknown</t>
         </is>
       </c>
       <c r="H169" s="2" t="inlineStr">
@@ -5856,22 +5861,22 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>No bedrooms unknown</t>
+          <t>Number of bedrooms</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>Set to true when counting units where bedroom number is unknown</t>
+          <t>The number of bedrooms in unit</t>
         </is>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -5895,12 +5900,12 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>Number of bedrooms</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>The number of bedrooms in unit</t>
+          <t>The number of units of that bedroom count</t>
         </is>
       </c>
       <c r="H171" s="2" t="inlineStr">
@@ -5910,7 +5915,7 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -5929,17 +5934,13 @@
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>Units per bedroom number[]</t>
-        </is>
-      </c>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
+          <t>Total units</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr"/>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>The number of units of that bedroom count</t>
+          <t>Total number of units</t>
         </is>
       </c>
       <c r="H172" s="2" t="inlineStr">
@@ -5949,7 +5950,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -5963,28 +5964,28 @@
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>Existing unit breakdown[]</t>
+          <t>Proposed unit breakdown[]</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>Total units</t>
+          <t>Units unknown</t>
         </is>
       </c>
       <c r="F173" s="2" t="inlineStr"/>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>Total number of units</t>
+          <t>Whether the number of units is unknown</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -6003,13 +6004,17 @@
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>Units unknown</t>
-        </is>
-      </c>
-      <c r="F174" s="2" t="inlineStr"/>
+          <t>Units per bedroom number[]</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>No bedrooms unknown</t>
+        </is>
+      </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>Whether the number of units is unknown</t>
+          <t>Set to true when counting units where bedroom number is unknown</t>
         </is>
       </c>
       <c r="H174" s="2" t="inlineStr">
@@ -6043,22 +6048,22 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>No bedrooms unknown</t>
+          <t>Number of bedrooms</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>Set to true when counting units where bedroom number is unknown</t>
+          <t>The number of bedrooms in unit</t>
         </is>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -6082,12 +6087,12 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>Number of bedrooms</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>The number of bedrooms in unit</t>
+          <t>The number of units of that bedroom count</t>
         </is>
       </c>
       <c r="H176" s="2" t="inlineStr">
@@ -6097,7 +6102,7 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -6116,17 +6121,13 @@
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>Units per bedroom number[]</t>
-        </is>
-      </c>
-      <c r="F177" s="2" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
+          <t>Total units</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr"/>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>The number of units of that bedroom count</t>
+          <t>Total number of units</t>
         </is>
       </c>
       <c r="H177" s="2" t="inlineStr">
@@ -6136,7 +6137,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -6145,23 +6146,15 @@
       <c r="B178" s="2" t="n"/>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Residential unit summary[]</t>
-        </is>
-      </c>
-      <c r="D178" s="2" t="inlineStr">
-        <is>
-          <t>Proposed unit breakdown[]</t>
-        </is>
-      </c>
-      <c r="E178" s="2" t="inlineStr">
-        <is>
-          <t>Total units</t>
-        </is>
-      </c>
+          <t>Total existing units</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr"/>
+      <c r="E178" s="2" t="inlineStr"/>
       <c r="F178" s="2" t="inlineStr"/>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>Total number of units</t>
+          <t>The total number of existing units</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr">
@@ -6171,7 +6164,7 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -6180,7 +6173,7 @@
       <c r="B179" s="2" t="n"/>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>Total existing units</t>
+          <t>Total proposed units</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr"/>
@@ -6188,7 +6181,7 @@
       <c r="F179" s="2" t="inlineStr"/>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>The total number of existing units</t>
+          <t>The total number of proposed units</t>
         </is>
       </c>
       <c r="H179" s="2" t="inlineStr">
@@ -6207,7 +6200,7 @@
       <c r="B180" s="2" t="n"/>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Total proposed units</t>
+          <t>Net change</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr"/>
@@ -6215,7 +6208,7 @@
       <c r="F180" s="2" t="inlineStr"/>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>The total number of proposed units</t>
+          <t>Calculated net change in units</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
@@ -6230,11 +6223,19 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n"/>
-      <c r="B181" s="2" t="n"/>
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>Site area</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>How big the site is including relevant measurements</t>
+        </is>
+      </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Net change</t>
+          <t>Site area in hectares</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr"/>
@@ -6242,7 +6243,7 @@
       <c r="F181" s="2" t="inlineStr"/>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>Calculated net change in units</t>
+          <t>The size of the site in hectares</t>
         </is>
       </c>
       <c r="H181" s="2" t="inlineStr">
@@ -6257,19 +6258,11 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="inlineStr">
-        <is>
-          <t>Site area</t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="inlineStr">
-        <is>
-          <t>How big the site is including relevant measurements</t>
-        </is>
-      </c>
+      <c r="A182" s="2" t="n"/>
+      <c r="B182" s="2" t="n"/>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>Site area in hectares</t>
+          <t>Site area provided by</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr"/>
@@ -6277,39 +6270,51 @@
       <c r="F182" s="2" t="inlineStr"/>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>The size of the site in hectares</t>
+          <t>Who provided the site area value</t>
         </is>
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n"/>
-      <c r="B183" s="2" t="n"/>
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>Site details</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>Where the proposed development will be built.</t>
+        </is>
+      </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>Site area provided by</t>
-        </is>
-      </c>
-      <c r="D183" s="2" t="inlineStr"/>
+          <t>Site locations[]</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>Site boundary</t>
+        </is>
+      </c>
       <c r="E183" s="2" t="inlineStr"/>
       <c r="F183" s="2" t="inlineStr"/>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>Who provided the site area value</t>
+          <t>Geometry of the site of the development, typically in GeoJSON format</t>
         </is>
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>wkt</t>
         </is>
       </c>
       <c r="I183" s="2" t="inlineStr">
@@ -6319,16 +6324,8 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="inlineStr">
-        <is>
-          <t>Site details</t>
-        </is>
-      </c>
-      <c r="B184" s="2" t="inlineStr">
-        <is>
-          <t>Where the proposed development will be built.</t>
-        </is>
-      </c>
+      <c r="A184" s="2" t="n"/>
+      <c r="B184" s="2" t="n"/>
       <c r="C184" s="2" t="inlineStr">
         <is>
           <t>Site locations[]</t>
@@ -6336,19 +6333,19 @@
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>Site boundary</t>
+          <t>Address Text</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr"/>
       <c r="F184" s="2" t="inlineStr"/>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>Geometry of the site of the development, typically in GeoJSON format</t>
+          <t>Flexible field for capturing addresses</t>
         </is>
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
-          <t>wkt</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I184" s="2" t="inlineStr">
@@ -6367,14 +6364,14 @@
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>Address Text</t>
+          <t>Postcode</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr"/>
       <c r="F185" s="2" t="inlineStr"/>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>The postal code</t>
         </is>
       </c>
       <c r="H185" s="2" t="inlineStr">
@@ -6398,19 +6395,19 @@
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>Postcode</t>
+          <t>Easting</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr"/>
       <c r="F186" s="2" t="inlineStr"/>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>The postal code</t>
+          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I186" s="2" t="inlineStr">
@@ -6429,14 +6426,14 @@
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>Easting</t>
+          <t>Northing</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr"/>
       <c r="F187" s="2" t="inlineStr"/>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
+          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H187" s="2" t="inlineStr">
@@ -6460,14 +6457,14 @@
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>Northing</t>
+          <t>Latitude</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr"/>
       <c r="F188" s="2" t="inlineStr"/>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
+          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H188" s="2" t="inlineStr">
@@ -6491,14 +6488,14 @@
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>Latitude</t>
+          <t>Longitude</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr"/>
       <c r="F189" s="2" t="inlineStr"/>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H189" s="2" t="inlineStr">
@@ -6522,19 +6519,19 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>Longitude</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr"/>
       <c r="F190" s="2" t="inlineStr"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>A text description providing details about the subject. For parking changes, this describes how the proposed works affect existing car parking arrangements.</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I190" s="2" t="inlineStr">
@@ -6553,14 +6550,14 @@
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>UPRNs[]</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr"/>
       <c r="F191" s="2" t="inlineStr"/>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>A text description providing details about the subject. For parking changes, this describes how the proposed works affect existing car parking arrangements.</t>
+          <t>Unique Property Reference Numbers (UPRNs) for properties within the site boundary</t>
         </is>
       </c>
       <c r="H191" s="2" t="inlineStr">
@@ -6575,50 +6572,46 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n"/>
-      <c r="B192" s="2" t="n"/>
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Site Visit Details</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>Information to help the planning authority arrange a site visit</t>
+        </is>
+      </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Site locations[]</t>
-        </is>
-      </c>
-      <c r="D192" s="2" t="inlineStr">
-        <is>
-          <t>UPRNs[]</t>
-        </is>
-      </c>
+          <t>Site seen from public area</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr"/>
       <c r="E192" s="2" t="inlineStr"/>
       <c r="F192" s="2" t="inlineStr"/>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>Unique Property Reference Numbers (UPRNs) for properties within the site boundary</t>
+          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="inlineStr">
-        <is>
-          <t>Site Visit Details</t>
-        </is>
-      </c>
-      <c r="B193" s="2" t="inlineStr">
-        <is>
-          <t>Information to help the planning authority arrange a site visit</t>
-        </is>
-      </c>
+      <c r="A193" s="2" t="n"/>
+      <c r="B193" s="2" t="n"/>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Site seen from public area</t>
+          <t>Site visit contact type</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr"/>
@@ -6626,12 +6619,12 @@
       <c r="F193" s="2" t="inlineStr"/>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
+          <t>Indicates who the authority should contact to arrange a site visit</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I193" s="2" t="inlineStr">
@@ -6645,7 +6638,7 @@
       <c r="B194" s="2" t="n"/>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Site visit contact type</t>
+          <t>Contact reference</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr"/>
@@ -6653,17 +6646,17 @@
       <c r="F194" s="2" t="inlineStr"/>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>Indicates who the authority should contact to arrange a site visit</t>
+          <t>The reference of the applicant or agent who should be contacted for site visits</t>
         </is>
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -6672,15 +6665,19 @@
       <c r="B195" s="2" t="n"/>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Contact reference</t>
-        </is>
-      </c>
-      <c r="D195" s="2" t="inlineStr"/>
+          <t>Other site visit contact</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>Full name</t>
+        </is>
+      </c>
       <c r="E195" s="2" t="inlineStr"/>
       <c r="F195" s="2" t="inlineStr"/>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>The reference of the applicant or agent who should be contacted for site visits</t>
+          <t>The complete name of a person</t>
         </is>
       </c>
       <c r="H195" s="2" t="inlineStr">
@@ -6690,7 +6687,7 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -6704,14 +6701,14 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>Full name</t>
+          <t>Phone number</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr"/>
       <c r="F196" s="2" t="inlineStr"/>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>The complete name of a person</t>
+          <t>A phone number</t>
         </is>
       </c>
       <c r="H196" s="2" t="inlineStr">
@@ -6735,14 +6732,14 @@
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>Phone number</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr"/>
       <c r="F197" s="2" t="inlineStr"/>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
       <c r="H197" s="2" t="inlineStr">
@@ -6757,28 +6754,32 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n"/>
-      <c r="B198" s="2" t="n"/>
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>Trade effluent</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>Details of any liquid waste produced by industial processes on the proposed site, and how it will be diposed of.</t>
+        </is>
+      </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Other site visit contact</t>
-        </is>
-      </c>
-      <c r="D198" s="2" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
+          <t>Disposal required</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr"/>
       <c r="E198" s="2" t="inlineStr"/>
       <c r="F198" s="2" t="inlineStr"/>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>The email address that can be used for electronic correspondence with the individual</t>
+          <t>Does the proposal involve the disposal of trade effluents or waste (true/false)</t>
         </is>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I198" s="2" t="inlineStr">
@@ -6788,19 +6789,11 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="inlineStr">
-        <is>
-          <t>Trade effluent</t>
-        </is>
-      </c>
-      <c r="B199" s="2" t="inlineStr">
-        <is>
-          <t>Details of any liquid waste produced by industial processes on the proposed site, and how it will be diposed of.</t>
-        </is>
-      </c>
+      <c r="A199" s="2" t="n"/>
+      <c r="B199" s="2" t="n"/>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>Disposal required</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr"/>
@@ -6808,26 +6801,34 @@
       <c r="F199" s="2" t="inlineStr"/>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t>Does the proposal involve the disposal of trade effluents or waste (true/false)</t>
+          <t>describe the nature, volume and means of disposal of trade effluents or waste</t>
         </is>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n"/>
-      <c r="B200" s="2" t="n"/>
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>Trees and hedges information</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>Details of trees and/or hedges that will be affected by the proposed development</t>
+        </is>
+      </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Trees on site</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr"/>
@@ -6835,34 +6836,26 @@
       <c r="F200" s="2" t="inlineStr"/>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>describe the nature, volume and means of disposal of trade effluents or waste</t>
+          <t>Whether trees or hedges are present on the proposed development site</t>
         </is>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="inlineStr">
-        <is>
-          <t>Trees and hedges information</t>
-        </is>
-      </c>
-      <c r="B201" s="2" t="inlineStr">
-        <is>
-          <t>Details of trees and/or hedges that will be affected by the proposed development</t>
-        </is>
-      </c>
+      <c r="A201" s="2" t="n"/>
+      <c r="B201" s="2" t="n"/>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>Trees on site</t>
+          <t>Trees on adjacent land</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr"/>
@@ -6870,7 +6863,7 @@
       <c r="F201" s="2" t="inlineStr"/>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>Whether trees or hedges are present on the proposed development site</t>
+          <t>Whether trees or hedges on land adjacent to the proposed development site could influence the development or might be important as part of the local landscape character</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
@@ -6885,24 +6878,36 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n"/>
-      <c r="B202" s="2" t="n"/>
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>Vehicle parking</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Details of current parking facilities at the site and any changes that would be made by the proposed development.</t>
+        </is>
+      </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Trees on adjacent land</t>
-        </is>
-      </c>
-      <c r="D202" s="2" t="inlineStr"/>
+          <t>Parking spaces[]</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>Parking space type</t>
+        </is>
+      </c>
       <c r="E202" s="2" t="inlineStr"/>
       <c r="F202" s="2" t="inlineStr"/>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>Whether trees or hedges on land adjacent to the proposed development site could influence the development or might be important as part of the local landscape character</t>
+          <t>Type of parking space or vehicle type</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I202" s="2" t="inlineStr">
@@ -6912,16 +6917,8 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="inlineStr">
-        <is>
-          <t>Vehicle parking</t>
-        </is>
-      </c>
-      <c r="B203" s="2" t="inlineStr">
-        <is>
-          <t>Details of current parking facilities at the site and any changes that would be made by the proposed development.</t>
-        </is>
-      </c>
+      <c r="A203" s="2" t="n"/>
+      <c r="B203" s="2" t="n"/>
       <c r="C203" s="2" t="inlineStr">
         <is>
           <t>Parking spaces[]</t>
@@ -6929,24 +6926,24 @@
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>Parking space type</t>
+          <t>Vehicle type other</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr"/>
       <c r="F203" s="2" t="inlineStr"/>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>Type of parking space or vehicle type</t>
+          <t>Vehicle type when parking space type is 'other'</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -6960,24 +6957,24 @@
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>Vehicle type other</t>
+          <t>Total existing</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr"/>
       <c r="F204" s="2" t="inlineStr"/>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>Vehicle type when parking space type is 'other'</t>
+          <t>Total number of existing parking spaces</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -6991,14 +6988,14 @@
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>Total existing</t>
+          <t>Total proposed</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr"/>
       <c r="F205" s="2" t="inlineStr"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>Total number of existing parking spaces</t>
+          <t>Total number of proposed parking spaces</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
@@ -7022,14 +7019,14 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>Total proposed</t>
+          <t>Difference in spaces</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr"/>
       <c r="F206" s="2" t="inlineStr"/>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>Total number of proposed parking spaces</t>
+          <t>Net change in parking spaces (proposed minus existing)</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
@@ -7044,28 +7041,32 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n"/>
-      <c r="B207" s="2" t="n"/>
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>Waste storage and collection</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>Any waste storage or recycling arrangements are in place, such as waste storage areas</t>
+        </is>
+      </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Parking spaces[]</t>
-        </is>
-      </c>
-      <c r="D207" s="2" t="inlineStr">
-        <is>
-          <t>Difference in spaces</t>
-        </is>
-      </c>
+          <t>Needs waste storage area</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr"/>
       <c r="E207" s="2" t="inlineStr"/>
       <c r="F207" s="2" t="inlineStr"/>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>Net change in parking spaces (proposed minus existing)</t>
+          <t>Does the proposal require a waste storage area</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I207" s="2" t="inlineStr">
@@ -7075,19 +7076,11 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="inlineStr">
-        <is>
-          <t>Waste storage and collection</t>
-        </is>
-      </c>
-      <c r="B208" s="2" t="inlineStr">
-        <is>
-          <t>Any waste storage or recycling arrangements are in place, such as waste storage areas</t>
-        </is>
-      </c>
+      <c r="A208" s="2" t="n"/>
+      <c r="B208" s="2" t="n"/>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Needs waste storage area</t>
+          <t>Waste storage area details</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr"/>
@@ -7095,17 +7088,17 @@
       <c r="F208" s="2" t="inlineStr"/>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>Does the proposal require a waste storage area</t>
+          <t>Details of the waste storage area including location, size, design and access arrangements</t>
         </is>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -7114,7 +7107,7 @@
       <c r="B209" s="2" t="n"/>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Waste storage area details</t>
+          <t>Separate recycling arrangements</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr"/>
@@ -7122,17 +7115,17 @@
       <c r="F209" s="2" t="inlineStr"/>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>Details of the waste storage area including location, size, design and access arrangements</t>
+          <t>Does the proposal include separate recycling arrangements</t>
         </is>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -7141,7 +7134,7 @@
       <c r="B210" s="2" t="n"/>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Separate recycling arrangements</t>
+          <t>Separate recycling arrangements details</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr"/>
@@ -7149,42 +7142,15 @@
       <c r="F210" s="2" t="inlineStr"/>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>Does the proposal include separate recycling arrangements</t>
+          <t>Details of the recycling arrangements including types of materials, collection methods and storage facilities</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I210" s="2" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" s="2" t="n"/>
-      <c r="B211" s="2" t="n"/>
-      <c r="C211" s="2" t="inlineStr">
-        <is>
-          <t>Separate recycling arrangements details</t>
-        </is>
-      </c>
-      <c r="D211" s="2" t="inlineStr"/>
-      <c r="E211" s="2" t="inlineStr"/>
-      <c r="F211" s="2" t="inlineStr"/>
-      <c r="G211" s="2" t="inlineStr">
-        <is>
-          <t>Details of the recycling arrangements including types of materials, collection methods and storage facilities</t>
-        </is>
-      </c>
-      <c r="H211" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="I211" s="2" t="inlineStr">
         <is>
           <t>MAY</t>
         </is>
@@ -7193,65 +7159,65 @@
   </sheetData>
   <mergeCells count="62">
     <mergeCell ref="B97:B100"/>
+    <mergeCell ref="A158:A164"/>
+    <mergeCell ref="A207:A210"/>
     <mergeCell ref="A115:A126"/>
-    <mergeCell ref="B193:B198"/>
     <mergeCell ref="B65:B67"/>
     <mergeCell ref="B64"/>
-    <mergeCell ref="A147:A158"/>
+    <mergeCell ref="A183:A191"/>
     <mergeCell ref="B68:B70"/>
     <mergeCell ref="A47:A49"/>
     <mergeCell ref="A25:A28"/>
-    <mergeCell ref="A203:A207"/>
-    <mergeCell ref="B182:B183"/>
-    <mergeCell ref="B208:B211"/>
+    <mergeCell ref="B147:B157"/>
     <mergeCell ref="B93:B96"/>
     <mergeCell ref="A41:A46"/>
     <mergeCell ref="A68:A70"/>
     <mergeCell ref="B2:B18"/>
     <mergeCell ref="B71:B76"/>
-    <mergeCell ref="A208:A211"/>
     <mergeCell ref="A101:A107"/>
+    <mergeCell ref="B158:B164"/>
     <mergeCell ref="A77:A86"/>
-    <mergeCell ref="A184:A192"/>
+    <mergeCell ref="A198:A199"/>
     <mergeCell ref="A87:A92"/>
     <mergeCell ref="A64"/>
+    <mergeCell ref="A202:A206"/>
     <mergeCell ref="B108:B114"/>
+    <mergeCell ref="A165:A180"/>
+    <mergeCell ref="B183:B191"/>
     <mergeCell ref="B142:B146"/>
-    <mergeCell ref="B166:B181"/>
-    <mergeCell ref="A159:A165"/>
     <mergeCell ref="B47:B49"/>
     <mergeCell ref="A37:A40"/>
-    <mergeCell ref="A193:A198"/>
+    <mergeCell ref="A147:A157"/>
+    <mergeCell ref="B181:B182"/>
     <mergeCell ref="B50:B63"/>
     <mergeCell ref="B115:B126"/>
     <mergeCell ref="A142:A146"/>
     <mergeCell ref="A71:A76"/>
     <mergeCell ref="B77:B86"/>
+    <mergeCell ref="A192:A197"/>
+    <mergeCell ref="B198:B199"/>
     <mergeCell ref="A97:A100"/>
-    <mergeCell ref="B201:B202"/>
     <mergeCell ref="B87:B92"/>
+    <mergeCell ref="A200:A201"/>
     <mergeCell ref="A2:A18"/>
     <mergeCell ref="B29:B36"/>
     <mergeCell ref="B37:B40"/>
     <mergeCell ref="A65:A67"/>
-    <mergeCell ref="B203:B207"/>
+    <mergeCell ref="B165:B180"/>
     <mergeCell ref="B19:B24"/>
-    <mergeCell ref="B159:B165"/>
-    <mergeCell ref="A199:A200"/>
-    <mergeCell ref="A166:A181"/>
+    <mergeCell ref="A181:A182"/>
+    <mergeCell ref="B202:B206"/>
     <mergeCell ref="B127:B141"/>
     <mergeCell ref="A93:A96"/>
-    <mergeCell ref="B184:B192"/>
-    <mergeCell ref="B147:B158"/>
+    <mergeCell ref="B207:B210"/>
     <mergeCell ref="A50:A63"/>
-    <mergeCell ref="A201:A202"/>
+    <mergeCell ref="B192:B197"/>
     <mergeCell ref="A29:A36"/>
-    <mergeCell ref="A182:A183"/>
+    <mergeCell ref="B200:B201"/>
     <mergeCell ref="B25:B28"/>
     <mergeCell ref="A19:A24"/>
     <mergeCell ref="A108:A114"/>
     <mergeCell ref="B101:B107"/>
-    <mergeCell ref="B199:B200"/>
     <mergeCell ref="B41:B46"/>
     <mergeCell ref="A127:A141"/>
   </mergeCells>

</xml_diff>